<commit_message>
Updated VNM_grids_kan model - 2025-12-05 23:54
</commit_message>
<xml_diff>
--- a/VerveStacks_VNM_grids_kan/Sets-vervestacks.xlsx
+++ b/VerveStacks_VNM_grids_kan/Sets-vervestacks.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr updateLinks="never" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_VNM_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D8A54A1E-8CB0-47F9-8A78-FCC2E1834794}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C08B3ED0-C671-471E-ACB8-027C8A884341}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2940" yWindow="2940" windowWidth="21600" windowHeight="12682" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="VEDA_Sets-Comm" sheetId="2" r:id="rId1"/>
@@ -10211,7 +10211,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92C0BC25-B11E-48C2-913B-58A0DC1A1F9A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A128CC4-8AEB-4C18-8F87-23C3A2F1E2B6}">
   <dimension ref="B9:E1514"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated VNM_grids_kan model - 2025-12-06 20:03
</commit_message>
<xml_diff>
--- a/VerveStacks_VNM_grids_kan/Sets-vervestacks.xlsx
+++ b/VerveStacks_VNM_grids_kan/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_VNM_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C08B3ED0-C671-471E-ACB8-027C8A884341}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{44427C61-D31F-4F61-8BBE-C1CD4FC186D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -10211,7 +10211,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A128CC4-8AEB-4C18-8F87-23C3A2F1E2B6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A61D1265-6A68-4FB8-B872-F91A1B788C2C}">
   <dimension ref="B9:E1514"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated VNM_grids_kan model - 2025-12-11 11:05
</commit_message>
<xml_diff>
--- a/VerveStacks_VNM_grids_kan/Sets-vervestacks.xlsx
+++ b/VerveStacks_VNM_grids_kan/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_VNM_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{44427C61-D31F-4F61-8BBE-C1CD4FC186D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{04199B74-4130-4C71-9BB5-A77AC0DA82B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -10211,7 +10211,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A61D1265-6A68-4FB8-B872-F91A1B788C2C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F05BF3C-6BDA-4FDA-8D95-0ABCE5AD9722}">
   <dimension ref="B9:E1514"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated VNM_grids_kan model - 2025-12-12 14:07
</commit_message>
<xml_diff>
--- a/VerveStacks_VNM_grids_kan/Sets-vervestacks.xlsx
+++ b/VerveStacks_VNM_grids_kan/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_VNM_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{04199B74-4130-4C71-9BB5-A77AC0DA82B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CABAF218-D666-4913-8EA3-FE266D3443C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -10211,7 +10211,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F05BF3C-6BDA-4FDA-8D95-0ABCE5AD9722}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C80EB26-F994-4CC8-8941-19225BEE7E5E}">
   <dimension ref="B9:E1514"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>